<commit_message>
feat: add evaluation pipeline for sentence similarity models using MRR, Accuracy, and LLM-as-a-judge metrics
</commit_message>
<xml_diff>
--- a/modelo_sentence_similarity/embedding_comparison_results.xlsx
+++ b/modelo_sentence_similarity/embedding_comparison_results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,40 +441,45 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Total Tokens</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>RAM Proceso (MB)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Tiempo Chunking (s)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Tiempo Embedding (s)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>MRR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Top_1_Accuracy</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>Top_3_Accuracy</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Precision@3</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Recall@3</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>LLM_Judge_Score</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Eficiencia (MRR / T.Emb)</t>
         </is>
@@ -496,28 +501,31 @@
         <v>49</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0005</v>
+        <v>4240</v>
       </c>
       <c r="F2" t="n">
-        <v>0.52</v>
+        <v>2254.83</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8857</v>
+        <v>0.0009</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8571</v>
+        <v>0.54</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2857</v>
+        <v>0.8611</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8571</v>
+        <v>0.7778</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>0.8889</v>
       </c>
       <c r="L2" t="n">
-        <v>1.6897</v>
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1.5969</v>
       </c>
     </row>
     <row r="3">
@@ -536,28 +544,31 @@
         <v>61</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0002</v>
+        <v>5413</v>
       </c>
       <c r="F3" t="n">
-        <v>0.92</v>
+        <v>2260.33</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9258999999999999</v>
+        <v>0.0003</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>0.55</v>
       </c>
       <c r="I3" t="n">
-        <v>0.3333</v>
+        <v>0.7751</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>0.6667</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>0.8889</v>
       </c>
       <c r="L3" t="n">
-        <v>1.0091</v>
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1.408</v>
       </c>
     </row>
     <row r="4">
@@ -576,28 +587,31 @@
         <v>111</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0005999999999999999</v>
+        <v>9767</v>
       </c>
       <c r="F4" t="n">
-        <v>1.44</v>
+        <v>2279.92</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6643</v>
+        <v>0.0003</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9</v>
+        <v>0.93</v>
       </c>
       <c r="I4" t="n">
-        <v>0.3</v>
+        <v>0.3985</v>
       </c>
       <c r="J4" t="n">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="L4" t="n">
-        <v>0.4616</v>
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.4302</v>
       </c>
     </row>
     <row r="5">
@@ -616,28 +630,31 @@
         <v>23</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0004</v>
+        <v>4222</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5</v>
+        <v>2280.51</v>
       </c>
       <c r="G5" t="n">
-        <v>0.6443</v>
+        <v>0.0003</v>
       </c>
       <c r="H5" t="n">
-        <v>0.75</v>
+        <v>0.29</v>
       </c>
       <c r="I5" t="n">
-        <v>0.25</v>
+        <v>0.7778</v>
       </c>
       <c r="J5" t="n">
-        <v>0.75</v>
+        <v>0.6667</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>0.8889</v>
       </c>
       <c r="L5" t="n">
-        <v>1.2905</v>
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>2.6468</v>
       </c>
     </row>
     <row r="6">
@@ -656,28 +673,31 @@
         <v>26</v>
       </c>
       <c r="E6" t="n">
-        <v>0.001</v>
+        <v>4692</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4</v>
+        <v>2271</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6061</v>
+        <v>0.0003</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7</v>
+        <v>0.32</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2333</v>
+        <v>0.6792</v>
       </c>
       <c r="J6" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="L6" t="n">
-        <v>1.5249</v>
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>2.0956</v>
       </c>
     </row>
     <row r="7">
@@ -696,28 +716,31 @@
         <v>31</v>
       </c>
       <c r="E7" t="n">
+        <v>5682</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2285.39</v>
+      </c>
+      <c r="G7" t="n">
         <v>0.0002</v>
       </c>
-      <c r="F7" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.5407</v>
-      </c>
       <c r="H7" t="n">
-        <v>0.5</v>
+        <v>0.38</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1667</v>
+        <v>0.4833</v>
       </c>
       <c r="J7" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="L7" t="n">
-        <v>1.3171</v>
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1.2645</v>
       </c>
     </row>
     <row r="8">
@@ -736,28 +759,31 @@
         <v>16</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0002</v>
+        <v>4242</v>
       </c>
       <c r="F8" t="n">
-        <v>0.36</v>
+        <v>2293.77</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5958</v>
+        <v>0.0003</v>
       </c>
       <c r="H8" t="n">
-        <v>0.75</v>
+        <v>0.23</v>
       </c>
       <c r="I8" t="n">
-        <v>0.25</v>
+        <v>0.6212</v>
       </c>
       <c r="J8" t="n">
-        <v>0.75</v>
+        <v>0.4444</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>0.8889</v>
       </c>
       <c r="L8" t="n">
-        <v>1.6477</v>
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2.7535</v>
       </c>
     </row>
     <row r="9">
@@ -776,28 +802,31 @@
         <v>16</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0003</v>
+        <v>4530</v>
       </c>
       <c r="F9" t="n">
-        <v>0.46</v>
+        <v>2296.12</v>
       </c>
       <c r="G9" t="n">
-        <v>0.791</v>
+        <v>0.0002</v>
       </c>
       <c r="H9" t="n">
-        <v>0.9</v>
+        <v>0.22</v>
       </c>
       <c r="I9" t="n">
-        <v>0.3</v>
+        <v>0.5673</v>
       </c>
       <c r="J9" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L9" t="n">
-        <v>1.7365</v>
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2.6386</v>
       </c>
     </row>
     <row r="10">
@@ -816,28 +845,31 @@
         <v>18</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0004</v>
+        <v>5080</v>
       </c>
       <c r="F10" t="n">
-        <v>0.33</v>
+        <v>2293.98</v>
       </c>
       <c r="G10" t="n">
-        <v>0.3046</v>
+        <v>0.0003</v>
       </c>
       <c r="H10" t="n">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1333</v>
+        <v>0.6348</v>
       </c>
       <c r="J10" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="L10" t="n">
-        <v>0.9104</v>
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2.4947</v>
       </c>
     </row>
     <row r="11">
@@ -856,28 +888,31 @@
         <v>49</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0007</v>
+        <v>4240</v>
       </c>
       <c r="F11" t="n">
-        <v>0.97</v>
+        <v>2297</v>
       </c>
       <c r="G11" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.8889</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.7778</v>
+      </c>
+      <c r="K11" t="n">
         <v>1</v>
       </c>
-      <c r="H11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0.3333</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
       <c r="L11" t="n">
-        <v>1.0303</v>
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1.8747</v>
       </c>
     </row>
     <row r="12">
@@ -896,28 +931,31 @@
         <v>61</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0008</v>
+        <v>5413</v>
       </c>
       <c r="F12" t="n">
-        <v>0.7</v>
+        <v>2294.29</v>
       </c>
       <c r="G12" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.8519</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.7778</v>
+      </c>
+      <c r="K12" t="n">
         <v>1</v>
       </c>
-      <c r="H12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0.3333</v>
-      </c>
-      <c r="J12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
       <c r="L12" t="n">
-        <v>1.4199</v>
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1.4097</v>
       </c>
     </row>
     <row r="13">
@@ -936,28 +974,31 @@
         <v>111</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0003</v>
+        <v>9767</v>
       </c>
       <c r="F13" t="n">
-        <v>1.24</v>
+        <v>2308.36</v>
       </c>
       <c r="G13" t="n">
-        <v>0.7333</v>
+        <v>0.0005</v>
       </c>
       <c r="H13" t="n">
         <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>0.3333</v>
+        <v>0.6083</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="L13" t="n">
-        <v>0.5937</v>
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.6056</v>
       </c>
     </row>
     <row r="14">
@@ -976,28 +1017,31 @@
         <v>23</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0009</v>
+        <v>4222</v>
       </c>
       <c r="F14" t="n">
+        <v>2318.47</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H14" t="n">
         <v>0.54</v>
       </c>
-      <c r="G14" t="n">
-        <v>0.8125</v>
-      </c>
-      <c r="H14" t="n">
-        <v>1</v>
-      </c>
       <c r="I14" t="n">
-        <v>0.3333</v>
+        <v>0.8519</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>0.7778</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>0.8889</v>
       </c>
       <c r="L14" t="n">
-        <v>1.5051</v>
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1.5674</v>
       </c>
     </row>
     <row r="15">
@@ -1016,28 +1060,31 @@
         <v>26</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0005999999999999999</v>
+        <v>4692</v>
       </c>
       <c r="F15" t="n">
-        <v>0.6899999999999999</v>
+        <v>2389.68</v>
       </c>
       <c r="G15" t="n">
-        <v>0.8</v>
+        <v>0.0002</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>0.62</v>
       </c>
       <c r="I15" t="n">
-        <v>0.3333</v>
+        <v>0.8167</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="L15" t="n">
-        <v>1.1666</v>
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1.307</v>
       </c>
     </row>
     <row r="16">
@@ -1056,28 +1103,31 @@
         <v>31</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0005</v>
+        <v>5682</v>
       </c>
       <c r="F16" t="n">
-        <v>0.95</v>
+        <v>2351.66</v>
       </c>
       <c r="G16" t="n">
-        <v>0.87</v>
+        <v>0.0004</v>
       </c>
       <c r="H16" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K16" t="n">
         <v>0.9</v>
       </c>
-      <c r="I16" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
       <c r="L16" t="n">
-        <v>0.9169</v>
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>1.0071</v>
       </c>
     </row>
     <row r="17">
@@ -1096,28 +1146,31 @@
         <v>16</v>
       </c>
       <c r="E17" t="n">
+        <v>4242</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2391.64</v>
+      </c>
+      <c r="G17" t="n">
         <v>0.0003</v>
       </c>
-      <c r="F17" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0.875</v>
-      </c>
       <c r="H17" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.8889</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.7778</v>
+      </c>
+      <c r="K17" t="n">
         <v>1</v>
       </c>
-      <c r="I17" t="n">
-        <v>0.3333</v>
-      </c>
-      <c r="J17" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
       <c r="L17" t="n">
-        <v>1.4549</v>
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>1.5826</v>
       </c>
     </row>
     <row r="18">
@@ -1136,28 +1189,31 @@
         <v>16</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0003</v>
+        <v>4530</v>
       </c>
       <c r="F18" t="n">
-        <v>0.63</v>
+        <v>2399.36</v>
       </c>
       <c r="G18" t="n">
-        <v>0.95</v>
+        <v>0.0002</v>
       </c>
       <c r="H18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.8167</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K18" t="n">
         <v>1</v>
       </c>
-      <c r="I18" t="n">
-        <v>0.3333</v>
-      </c>
-      <c r="J18" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
       <c r="L18" t="n">
-        <v>1.5103</v>
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>1.4726</v>
       </c>
     </row>
     <row r="19">
@@ -1176,28 +1232,31 @@
         <v>18</v>
       </c>
       <c r="E19" t="n">
+        <v>5080</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2356.25</v>
+      </c>
+      <c r="G19" t="n">
         <v>0.0004</v>
       </c>
-      <c r="F19" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.9</v>
-      </c>
       <c r="H19" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K19" t="n">
         <v>1</v>
       </c>
-      <c r="I19" t="n">
-        <v>0.3333</v>
-      </c>
-      <c r="J19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
       <c r="L19" t="n">
-        <v>1.2482</v>
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>1.3017</v>
       </c>
     </row>
     <row r="20">
@@ -1216,28 +1275,31 @@
         <v>49</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0008</v>
+        <v>4617</v>
       </c>
       <c r="F20" t="n">
-        <v>0.97</v>
+        <v>2435.96</v>
       </c>
       <c r="G20" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="I20" t="n">
         <v>1</v>
-      </c>
-      <c r="H20" t="n">
-        <v>1</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0.3333</v>
       </c>
       <c r="J20" t="n">
         <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>1.0288</v>
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>1.0083</v>
       </c>
     </row>
     <row r="21">
@@ -1256,28 +1318,31 @@
         <v>61</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0004</v>
+        <v>5919</v>
       </c>
       <c r="F21" t="n">
-        <v>1.25</v>
+        <v>2411.76</v>
       </c>
       <c r="G21" t="n">
-        <v>0.9444</v>
+        <v>0.0003</v>
       </c>
       <c r="H21" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.8704</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.7778</v>
+      </c>
+      <c r="K21" t="n">
         <v>1</v>
       </c>
-      <c r="I21" t="n">
-        <v>0.3333</v>
-      </c>
-      <c r="J21" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
       <c r="L21" t="n">
-        <v>0.7568</v>
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.7013</v>
       </c>
     </row>
     <row r="22">
@@ -1296,28 +1361,31 @@
         <v>111</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0004</v>
+        <v>10632</v>
       </c>
       <c r="F22" t="n">
-        <v>2.28</v>
+        <v>2422.16</v>
       </c>
       <c r="G22" t="n">
-        <v>0.55</v>
+        <v>0.0005</v>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>2.12</v>
       </c>
       <c r="I22" t="n">
-        <v>0.3333</v>
+        <v>0.5144</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="L22" t="n">
-        <v>0.2413</v>
+        <v>0</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.2429</v>
       </c>
     </row>
     <row r="23">
@@ -1336,28 +1404,31 @@
         <v>23</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0003</v>
+        <v>4600</v>
       </c>
       <c r="F23" t="n">
-        <v>0.62</v>
+        <v>2440.02</v>
       </c>
       <c r="G23" t="n">
-        <v>0.599</v>
+        <v>0.0004</v>
       </c>
       <c r="H23" t="n">
-        <v>0.5</v>
+        <v>0.54</v>
       </c>
       <c r="I23" t="n">
-        <v>0.1667</v>
+        <v>0.9258999999999999</v>
       </c>
       <c r="J23" t="n">
-        <v>0.5</v>
+        <v>0.8889</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>0.9713000000000001</v>
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>1.7223</v>
       </c>
     </row>
     <row r="24">
@@ -1376,28 +1447,31 @@
         <v>26</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0008</v>
+        <v>5106</v>
       </c>
       <c r="F24" t="n">
-        <v>0.66</v>
+        <v>2438.07</v>
       </c>
       <c r="G24" t="n">
-        <v>0.6811</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="H24" t="n">
-        <v>0.7</v>
+        <v>0.59</v>
       </c>
       <c r="I24" t="n">
-        <v>0.2333</v>
+        <v>0.77</v>
       </c>
       <c r="J24" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="L24" t="n">
-        <v>1.026</v>
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>1.3085</v>
       </c>
     </row>
     <row r="25">
@@ -1416,28 +1490,31 @@
         <v>31</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0004</v>
+        <v>6174</v>
       </c>
       <c r="F25" t="n">
-        <v>0.84</v>
+        <v>2424.19</v>
       </c>
       <c r="G25" t="n">
-        <v>0.4982</v>
+        <v>0.0003</v>
       </c>
       <c r="H25" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.6183</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K25" t="n">
         <v>0.6</v>
       </c>
-      <c r="I25" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
       <c r="L25" t="n">
-        <v>0.5903</v>
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.855</v>
       </c>
     </row>
     <row r="26">
@@ -1456,28 +1533,31 @@
         <v>16</v>
       </c>
       <c r="E26" t="n">
-        <v>0.0005</v>
+        <v>4621</v>
       </c>
       <c r="F26" t="n">
-        <v>0.42</v>
+        <v>2441.96</v>
       </c>
       <c r="G26" t="n">
-        <v>0.4562</v>
+        <v>0.0008</v>
       </c>
       <c r="H26" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="I26" t="n">
-        <v>0.1667</v>
+        <v>0.7566000000000001</v>
       </c>
       <c r="J26" t="n">
-        <v>0.5</v>
+        <v>0.6667</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>0.7778</v>
       </c>
       <c r="L26" t="n">
-        <v>1.0796</v>
+        <v>0</v>
+      </c>
+      <c r="M26" t="n">
+        <v>1.4146</v>
       </c>
     </row>
     <row r="27">
@@ -1496,28 +1576,31 @@
         <v>16</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0004</v>
+        <v>4952</v>
       </c>
       <c r="F27" t="n">
-        <v>0.41</v>
+        <v>2423.64</v>
       </c>
       <c r="G27" t="n">
-        <v>0.6861</v>
+        <v>0.0005</v>
       </c>
       <c r="H27" t="n">
-        <v>0.8</v>
+        <v>0.39</v>
       </c>
       <c r="I27" t="n">
-        <v>0.2667</v>
+        <v>0.5798</v>
       </c>
       <c r="J27" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L27" t="n">
-        <v>1.6701</v>
+        <v>0</v>
+      </c>
+      <c r="M27" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="28">
@@ -1536,28 +1619,31 @@
         <v>18</v>
       </c>
       <c r="E28" t="n">
-        <v>0.0019</v>
+        <v>5527</v>
       </c>
       <c r="F28" t="n">
-        <v>0.46</v>
+        <v>2461.35</v>
       </c>
       <c r="G28" t="n">
-        <v>0.3848</v>
+        <v>0.0003</v>
       </c>
       <c r="H28" t="n">
-        <v>0.4</v>
+        <v>0.43</v>
       </c>
       <c r="I28" t="n">
-        <v>0.1333</v>
+        <v>0.58</v>
       </c>
       <c r="J28" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L28" t="n">
-        <v>0.8421999999999999</v>
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
+        <v>1.3421</v>
       </c>
     </row>
   </sheetData>
@@ -1571,7 +1657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1597,40 +1683,45 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Total Tokens</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>RAM Proceso (MB)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Tiempo Chunking (s)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Tiempo Embedding (s)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>MRR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Top_1_Accuracy</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>Top_3_Accuracy</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Precision@3</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Recall@3</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>LLM_Judge_Score</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Eficiencia (MRR / T.Emb)</t>
         </is>
@@ -1639,41 +1730,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>intfloat/multilingual-e5-small</t>
+          <t>sentence-transformers/distiluse-base-multilingual-cased-v1</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>500</v>
       </c>
       <c r="C2" t="n">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="D2" t="n">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0008</v>
+        <v>4617</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7</v>
+        <v>2435.96</v>
       </c>
       <c r="G2" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="I2" t="n">
         <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.3333</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>1.4199</v>
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1.0083</v>
       </c>
     </row>
   </sheetData>
@@ -1687,7 +1781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1716,6 +1810,16 @@
           <t>Tiempo Embedding (s)</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Total Tokens</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>RAM Proceso (MB)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1724,16 +1828,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8823111111111112</v>
+        <v>0.8103666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9888888888888889</v>
+        <v>0.9543222222222223</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7822222222222223</v>
+        <v>0.6344444444444445</v>
+      </c>
+      <c r="F2" t="n">
+        <v>5318.666666666667</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2399.36</v>
       </c>
     </row>
     <row r="3">
@@ -1743,16 +1853,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.6444222222222222</v>
+        <v>0.7350444444444445</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.7864222222222222</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8788888888888889</v>
+        <v>0.8388888888888889</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5794.222222222223</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2461.35</v>
       </c>
     </row>
     <row r="4">
@@ -1762,16 +1878,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.6620444444444444</v>
+        <v>0.6442555555555556</v>
       </c>
       <c r="C4" t="n">
-        <v>0.750788888888889</v>
+        <v>0.7839555555555555</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.5933333333333333</v>
+        <v>0.4122222222222222</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5318.666666666667</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2296.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>